<commit_message>
refactor: enum ItemType의 순서를 id 순서로 변경
</commit_message>
<xml_diff>
--- a/Assets/Project/Csv/Item/ItemTable.xlsx
+++ b/Assets/Project/Csv/Item/ItemTable.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ycjun\OneDrive\문서\Projects\Git\Dairy Farm\Assets\Project\Csv\Item\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB274F4-4D59-4AA2-9CCF-A0BE8B532B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A31B1A1-2029-4DC6-AC5A-1B09DDF97C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Database" sheetId="1" r:id="rId1"/>
+    <sheet name="enum ItemType" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -156,22 +157,6 @@
     <t>Frog</t>
   </si>
   <si>
-    <t>대충</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>아무거나</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>넣으</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>시오</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>물뿌리개</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -181,6 +166,22 @@
   </si>
   <si>
     <t>더 많은 물을 담을 수 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>생선</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>입니</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>다</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -640,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.625" style="1" bestFit="1" customWidth="1"/>
@@ -652,7 +653,7 @@
     <col min="8" max="8" width="15.25" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>22</v>
       </c>
@@ -671,14 +672,8 @@
       <c r="F1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -695,21 +690,15 @@
         <v>100</v>
       </c>
       <c r="F2" s="2">
-        <v>2</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>17</v>
@@ -721,24 +710,18 @@
         <v>100</v>
       </c>
       <c r="F3" s="2">
-        <v>2</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
@@ -747,12 +730,10 @@
         <v>200</v>
       </c>
       <c r="F4" s="2">
-        <v>2</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>20</v>
       </c>
@@ -769,16 +750,10 @@
         <v>100</v>
       </c>
       <c r="F5" s="2">
-        <v>2</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>30</v>
       </c>
@@ -795,10 +770,10 @@
         <v>100</v>
       </c>
       <c r="F6" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>100</v>
       </c>
@@ -818,7 +793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>110</v>
       </c>
@@ -838,7 +813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>120</v>
       </c>
@@ -858,7 +833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>130</v>
       </c>
@@ -878,7 +853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>200</v>
       </c>
@@ -898,7 +873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>1000</v>
       </c>
@@ -915,10 +890,10 @@
         <v>0</v>
       </c>
       <c r="F12" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>1100</v>
       </c>
@@ -935,10 +910,10 @@
         <v>0</v>
       </c>
       <c r="F13" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>1200</v>
       </c>
@@ -955,10 +930,10 @@
         <v>0</v>
       </c>
       <c r="F14" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>1300</v>
       </c>
@@ -975,10 +950,10 @@
         <v>0</v>
       </c>
       <c r="F15" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>2000</v>
       </c>
@@ -986,7 +961,7 @@
         <v>36</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D16" s="10">
         <v>99</v>
@@ -995,7 +970,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1006,7 +981,7 @@
         <v>37</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D17" s="10">
         <v>99</v>
@@ -1015,7 +990,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1026,7 +1001,7 @@
         <v>38</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D18" s="10">
         <v>99</v>
@@ -1035,7 +1010,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1046,7 +1021,7 @@
         <v>39</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D19" s="10">
         <v>99</v>
@@ -1055,7 +1030,54 @@
         <v>4</v>
       </c>
       <c r="F19" s="5">
-        <v>0</v>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B24F2156-F927-4594-8663-BE0E26A1014A}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="7">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>